<commit_message>
Updated TUR_grids_kan50 model - 2026-09-28 21:24
</commit_message>
<xml_diff>
--- a/VerveStacks_TUR_grids_kan50/Sets-vervestacks.xlsx
+++ b/VerveStacks_TUR_grids_kan50/Sets-vervestacks.xlsx
@@ -2,26 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
-  <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_TUR_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BD668D-77E7-4D6A-AFFA-3BC28A66C62E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96451FFB-E1DC-4AA6-8508-2BFFBBFBA4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="11422" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12772" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
-    <sheet name="geo_sets" sheetId="5" r:id="rId2"/>
-    <sheet name="VEDA_Sets-Proc" sheetId="4" r:id="rId3"/>
+    <sheet name="VEDA_Sets-Comm" sheetId="1" r:id="rId1"/>
+    <sheet name="geo_sets" sheetId="2" r:id="rId2"/>
+    <sheet name="VEDA_Sets-Proc" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -40,6 +37,129 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="373">
   <si>
+    <t>~TFM_Csets</t>
+  </si>
+  <si>
+    <t>CSET_SET</t>
+  </si>
+  <si>
+    <t>CSET_CN</t>
+  </si>
+  <si>
+    <t>CSET_CD</t>
+  </si>
+  <si>
+    <t>SetName</t>
+  </si>
+  <si>
+    <t>SetDesc</t>
+  </si>
+  <si>
+    <t>c_Pos_AndOr</t>
+  </si>
+  <si>
+    <t>c_Neg_AndOr</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>e*spv*</t>
+  </si>
+  <si>
+    <t>Solar elec</t>
+  </si>
+  <si>
+    <t>e*won*,e*wof*</t>
+  </si>
+  <si>
+    <t>Wind elec</t>
+  </si>
+  <si>
+    <t>coal,gas,oil</t>
+  </si>
+  <si>
+    <t>fossil</t>
+  </si>
+  <si>
+    <t>geothermal,hydro,solar,wind</t>
+  </si>
+  <si>
+    <t>renewable</t>
+  </si>
+  <si>
+    <t>bioenergy</t>
+  </si>
+  <si>
+    <t>hydrogen</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>ELC,e[_]*</t>
+  </si>
+  <si>
+    <t>Electricity</t>
+  </si>
+  <si>
+    <t>elc_buildings</t>
+  </si>
+  <si>
+    <t>buildings</t>
+  </si>
+  <si>
+    <t>elc_industry</t>
+  </si>
+  <si>
+    <t>industry</t>
+  </si>
+  <si>
+    <t>elc_transport</t>
+  </si>
+  <si>
+    <t>transport</t>
+  </si>
+  <si>
+    <t>elc_roadtransport</t>
+  </si>
+  <si>
+    <t>EVs</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>co2captured,co2[_]*</t>
+  </si>
+  <si>
+    <t>CO2Captured</t>
+  </si>
+  <si>
+    <t>co2s[_]*</t>
+  </si>
+  <si>
+    <t>CO2Stored</t>
+  </si>
+  <si>
+    <t>~tfm_psets</t>
+  </si>
+  <si>
+    <t>setname</t>
+  </si>
+  <si>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>pset_ci</t>
+  </si>
+  <si>
+    <t>t_pos_andor</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
     <t>~TFM_Psets</t>
   </si>
   <si>
@@ -58,463 +178,340 @@
     <t>PSET_CO</t>
   </si>
   <si>
-    <t>SetName</t>
-  </si>
-  <si>
-    <t>SetDesc</t>
-  </si>
-  <si>
     <t>T_Pos_AndOr</t>
   </si>
   <si>
     <t>T_Neg_AndOr</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>ELE</t>
   </si>
   <si>
-    <t>~TFM_Csets</t>
-  </si>
-  <si>
-    <t>CSET_SET</t>
-  </si>
-  <si>
-    <t>CSET_CN</t>
-  </si>
-  <si>
-    <t>CSET_CD</t>
-  </si>
-  <si>
-    <t>c_Pos_AndOr</t>
-  </si>
-  <si>
-    <t>c_Neg_AndOr</t>
+    <t>EP_GAS-CC*,EP_OIL-CC*,*gas_cc*,*gas_comb*,*ember</t>
+  </si>
+  <si>
+    <t>gas,elcnga,elcgas,oil,elco</t>
   </si>
   <si>
     <t>CCGT</t>
   </si>
   <si>
+    <t>Combined Cycle Gas Turbine</t>
+  </si>
+  <si>
+    <t>Ramp ~8%/min</t>
+  </si>
+  <si>
+    <t>EP_GAS-GT*,EP_OIL-GT*,*gas_turbine*,EN*CT*</t>
+  </si>
+  <si>
+    <t>OCGT</t>
+  </si>
+  <si>
+    <t>Open Cycle Gas Turbine (Peaker)</t>
+  </si>
+  <si>
+    <t>Ramp ~15%/min</t>
+  </si>
+  <si>
+    <t>EP_GAS-ST*,EP_OIL-ST*,*steam*</t>
+  </si>
+  <si>
+    <t>Gas_Oil_Steam</t>
+  </si>
+  <si>
+    <t>Gas/Oil Steam Turbine</t>
+  </si>
+  <si>
+    <t>EP_GAS-IC*,EP_OIL-IC*,*gas_engine*,*internal_comb*</t>
+  </si>
+  <si>
+    <t>Int_Comb</t>
+  </si>
+  <si>
+    <t>Internal Combustion Engine</t>
+  </si>
+  <si>
+    <t>EP_COA-ST*,EP_LIG-ST*,*-CFB*,*coal_st*,*coal_subcritical*</t>
+  </si>
+  <si>
+    <t>coal,elcco*</t>
+  </si>
+  <si>
+    <t>Subcrit_Coal</t>
+  </si>
+  <si>
     <t>Subcritical Coal</t>
   </si>
   <si>
+    <t>Ramp ~3%/min</t>
+  </si>
+  <si>
+    <t>EP_COA-SC*,EP_COA-USC*,EP_LIG-SC*,EP_LIG-USC*,*coal_sc*,*coal_usc*,*coal_supercritical*,*coal_ultrasupercritical*</t>
+  </si>
+  <si>
+    <t>Supercrit_Coal</t>
+  </si>
+  <si>
+    <t>Supercritical/Ultra-Supercritical Coal</t>
+  </si>
+  <si>
+    <t>Ramp ~4%/min</t>
+  </si>
+  <si>
+    <t>*-IGCC*,*coal_igcc*</t>
+  </si>
+  <si>
+    <t>IGCC</t>
+  </si>
+  <si>
+    <t>Integrated Gasification CC</t>
+  </si>
+  <si>
+    <t>CHP</t>
+  </si>
+  <si>
+    <t>CHP_Gas</t>
+  </si>
+  <si>
+    <t>Gas/Oil CHP</t>
+  </si>
+  <si>
+    <t>Same ramp as ELE counterpart</t>
+  </si>
+  <si>
+    <t>CHP_Coal</t>
+  </si>
+  <si>
+    <t>Coal CHP</t>
+  </si>
+  <si>
+    <t>bio*,elcb*</t>
+  </si>
+  <si>
+    <t>CHP_Bio</t>
+  </si>
+  <si>
+    <t>Biomass CHP</t>
+  </si>
+  <si>
+    <t>HPL</t>
+  </si>
+  <si>
+    <t>HOP_Gas</t>
+  </si>
+  <si>
+    <t>Gas/Oil Heat-Only Boiler</t>
+  </si>
+  <si>
+    <t>HOP_Bio</t>
+  </si>
+  <si>
+    <t>Biomass Heat-Only Boiler</t>
+  </si>
+  <si>
+    <t>-*HP*</t>
+  </si>
+  <si>
+    <t>elc,e[_]*</t>
+  </si>
+  <si>
+    <t>HOP_Elec</t>
+  </si>
+  <si>
+    <t>Electric Boiler (DH)</t>
+  </si>
+  <si>
+    <t>*HP*</t>
+  </si>
+  <si>
+    <t>Heat_Pump</t>
+  </si>
+  <si>
+    <t>Large-Scale Heat Pump</t>
+  </si>
+  <si>
+    <t>Bio_Power</t>
+  </si>
+  <si>
+    <t>Biomass Power (ELE)</t>
+  </si>
+  <si>
+    <t>ELE,CHP</t>
+  </si>
+  <si>
+    <t>elcs*,solar</t>
+  </si>
+  <si>
+    <t>Solar_Util</t>
+  </si>
+  <si>
+    <t>Solar Utility</t>
+  </si>
+  <si>
+    <t>elcwin,windon</t>
+  </si>
+  <si>
+    <t>Wind_Onshore</t>
+  </si>
+  <si>
+    <t>Wind Onshore</t>
+  </si>
+  <si>
+    <t>windoff</t>
+  </si>
+  <si>
+    <t>Wind_Offshore</t>
+  </si>
+  <si>
+    <t>Wind Offshore</t>
+  </si>
+  <si>
+    <t>elcgeo,geothermal</t>
+  </si>
+  <si>
+    <t>Geothermal</t>
+  </si>
+  <si>
+    <t>Geothermal Power</t>
+  </si>
+  <si>
+    <t>-*ror*</t>
+  </si>
+  <si>
+    <t>elchyd,hydro</t>
+  </si>
+  <si>
+    <t>Hydro_Dam</t>
+  </si>
+  <si>
+    <t>Hydro Dam</t>
+  </si>
+  <si>
+    <t>And</t>
+  </si>
+  <si>
+    <t>Or</t>
+  </si>
+  <si>
+    <t>*HYD-ROR*,*ror*</t>
+  </si>
+  <si>
+    <t>Hydro_RoR</t>
+  </si>
+  <si>
+    <t>Hydro Run-of-River</t>
+  </si>
+  <si>
+    <t>-*SMR*</t>
+  </si>
+  <si>
+    <t>elcnuc,nuclear</t>
+  </si>
+  <si>
+    <t>Nuclear_P</t>
+  </si>
+  <si>
+    <t>Nuclear (Conventional)</t>
+  </si>
+  <si>
+    <t>*SMR*</t>
+  </si>
+  <si>
+    <t>Nuclear_SMR</t>
+  </si>
+  <si>
+    <t>Nuclear SMR</t>
+  </si>
+  <si>
     <t>STG</t>
   </si>
   <si>
-    <t>IGCC</t>
+    <t>*HPS*,*hydro_ps*</t>
+  </si>
+  <si>
+    <t>Hydro_PS</t>
+  </si>
+  <si>
+    <t>Pumped Hydro Storage</t>
+  </si>
+  <si>
+    <t>*4h*,*8h*,*12h*,-*EV*</t>
+  </si>
+  <si>
+    <t>Batt_Util</t>
+  </si>
+  <si>
+    <t>Utility Battery Storage</t>
   </si>
   <si>
     <t>*EV*</t>
   </si>
   <si>
+    <t>Batt_EV</t>
+  </si>
+  <si>
+    <t>EV Battery</t>
+  </si>
+  <si>
+    <t>IRE</t>
+  </si>
+  <si>
+    <t>g[_]*</t>
+  </si>
+  <si>
+    <t>Grid</t>
+  </si>
+  <si>
+    <t>DMD</t>
+  </si>
+  <si>
+    <t>Demand</t>
+  </si>
+  <si>
+    <t>PRE</t>
+  </si>
+  <si>
+    <t>stepdown*</t>
+  </si>
+  <si>
+    <t>Transformers Dn</t>
+  </si>
+  <si>
+    <t>stepup*</t>
+  </si>
+  <si>
+    <t>Transformers Up</t>
+  </si>
+  <si>
+    <t>distr*</t>
+  </si>
+  <si>
+    <t>Aggregators</t>
+  </si>
+  <si>
+    <t>IMP*Z</t>
+  </si>
+  <si>
+    <t>DUMMY_IMP</t>
+  </si>
+  <si>
+    <t>distr_sol*</t>
+  </si>
+  <si>
+    <t>distr_won*</t>
+  </si>
+  <si>
+    <t>distr_wof*</t>
+  </si>
+  <si>
     <t>geothermal</t>
   </si>
   <si>
     <t>hydro</t>
   </si>
   <si>
-    <t>nuclear</t>
-  </si>
-  <si>
-    <t>And</t>
-  </si>
-  <si>
-    <t>Or</t>
-  </si>
-  <si>
-    <t>Grid</t>
-  </si>
-  <si>
-    <t>IRE</t>
-  </si>
-  <si>
-    <t>g[_]*</t>
-  </si>
-  <si>
-    <t>DMD</t>
-  </si>
-  <si>
-    <t>Demand</t>
-  </si>
-  <si>
-    <t>e*spv*</t>
-  </si>
-  <si>
-    <t>e*won*,e*wof*</t>
-  </si>
-  <si>
-    <t>bioenergy</t>
-  </si>
-  <si>
-    <t>hydrogen</t>
-  </si>
-  <si>
-    <t>elc_buildings</t>
-  </si>
-  <si>
-    <t>elc_industry</t>
-  </si>
-  <si>
-    <t>elc_transport</t>
-  </si>
-  <si>
-    <t>elc_roadtransport</t>
-  </si>
-  <si>
-    <t>co2</t>
-  </si>
-  <si>
-    <t>buildings</t>
-  </si>
-  <si>
-    <t>industry</t>
-  </si>
-  <si>
-    <t>transport</t>
-  </si>
-  <si>
-    <t>EVs</t>
-  </si>
-  <si>
-    <t>fossil</t>
-  </si>
-  <si>
-    <t>coal,gas,oil</t>
-  </si>
-  <si>
-    <t>geothermal,hydro,solar,wind</t>
-  </si>
-  <si>
-    <t>PRE</t>
-  </si>
-  <si>
-    <t>stepdown*</t>
-  </si>
-  <si>
-    <t>Nuclear SMR</t>
-  </si>
-  <si>
-    <t>*SMR*</t>
-  </si>
-  <si>
-    <t>-*SMR*</t>
-  </si>
-  <si>
-    <t>Hydro Dam</t>
-  </si>
-  <si>
-    <t>renewable</t>
-  </si>
-  <si>
-    <t>Solar elec</t>
-  </si>
-  <si>
-    <t>Wind elec</t>
-  </si>
-  <si>
-    <t>Aggregators</t>
-  </si>
-  <si>
-    <t>IMP*Z</t>
-  </si>
-  <si>
-    <t>DUMMY_IMP</t>
-  </si>
-  <si>
-    <t>stepup*</t>
-  </si>
-  <si>
-    <t>Transformers Up</t>
-  </si>
-  <si>
-    <t>Transformers Dn</t>
-  </si>
-  <si>
-    <t>windoff</t>
-  </si>
-  <si>
-    <t>distr*</t>
-  </si>
-  <si>
-    <t>ELE,CHP</t>
-  </si>
-  <si>
-    <t>distr_sol*</t>
-  </si>
-  <si>
-    <t>distr_won*</t>
-  </si>
-  <si>
-    <t>distr_wof*</t>
-  </si>
-  <si>
     <t>coal</t>
-  </si>
-  <si>
-    <t>*4h*,*8h*,*12h*,-*EV*</t>
-  </si>
-  <si>
-    <t>Combined Cycle Gas Turbine</t>
-  </si>
-  <si>
-    <t>Ramp ~8%/min</t>
-  </si>
-  <si>
-    <t>OCGT</t>
-  </si>
-  <si>
-    <t>Open Cycle Gas Turbine (Peaker)</t>
-  </si>
-  <si>
-    <t>Ramp ~15%/min</t>
-  </si>
-  <si>
-    <t>Gas_Oil_Steam</t>
-  </si>
-  <si>
-    <t>Gas/Oil Steam Turbine</t>
-  </si>
-  <si>
-    <t>Int_Comb</t>
-  </si>
-  <si>
-    <t>Internal Combustion Engine</t>
-  </si>
-  <si>
-    <t>Subcrit_Coal</t>
-  </si>
-  <si>
-    <t>Ramp ~3%/min</t>
-  </si>
-  <si>
-    <t>Supercrit_Coal</t>
-  </si>
-  <si>
-    <t>Supercritical/Ultra-Supercritical Coal</t>
-  </si>
-  <si>
-    <t>Ramp ~4%/min</t>
-  </si>
-  <si>
-    <t>*-IGCC*,*coal_igcc*</t>
-  </si>
-  <si>
-    <t>Integrated Gasification CC</t>
-  </si>
-  <si>
-    <t>CHP</t>
-  </si>
-  <si>
-    <t>CHP_Gas</t>
-  </si>
-  <si>
-    <t>Gas/Oil CHP</t>
-  </si>
-  <si>
-    <t>Same ramp as ELE counterpart</t>
-  </si>
-  <si>
-    <t>CHP_Coal</t>
-  </si>
-  <si>
-    <t>Coal CHP</t>
-  </si>
-  <si>
-    <t>CHP_Bio</t>
-  </si>
-  <si>
-    <t>Biomass CHP</t>
-  </si>
-  <si>
-    <t>HPL</t>
-  </si>
-  <si>
-    <t>HOP_Gas</t>
-  </si>
-  <si>
-    <t>Gas/Oil Heat-Only Boiler</t>
-  </si>
-  <si>
-    <t>HOP_Bio</t>
-  </si>
-  <si>
-    <t>Biomass Heat-Only Boiler</t>
-  </si>
-  <si>
-    <t>HOP_Elec</t>
-  </si>
-  <si>
-    <t>Electric Boiler (DH)</t>
-  </si>
-  <si>
-    <t>Heat_Pump</t>
-  </si>
-  <si>
-    <t>Large-Scale Heat Pump</t>
-  </si>
-  <si>
-    <t>Bio_Power</t>
-  </si>
-  <si>
-    <t>Biomass Power (ELE)</t>
-  </si>
-  <si>
-    <t>elcs*,solar</t>
-  </si>
-  <si>
-    <t>Solar_Util</t>
-  </si>
-  <si>
-    <t>Solar Utility</t>
-  </si>
-  <si>
-    <t>elcwin,windon</t>
-  </si>
-  <si>
-    <t>Wind_Onshore</t>
-  </si>
-  <si>
-    <t>Wind Onshore</t>
-  </si>
-  <si>
-    <t>Wind_Offshore</t>
-  </si>
-  <si>
-    <t>Wind Offshore</t>
-  </si>
-  <si>
-    <t>elcgeo,geothermal</t>
-  </si>
-  <si>
-    <t>Geothermal</t>
-  </si>
-  <si>
-    <t>Geothermal Power</t>
-  </si>
-  <si>
-    <t>elchyd,hydro</t>
-  </si>
-  <si>
-    <t>Hydro_Dam</t>
-  </si>
-  <si>
-    <t>*HYD-ROR*,*ror*</t>
-  </si>
-  <si>
-    <t>Hydro_RoR</t>
-  </si>
-  <si>
-    <t>Hydro Run-of-River</t>
-  </si>
-  <si>
-    <t>elcnuc,nuclear</t>
-  </si>
-  <si>
-    <t>Nuclear (Conventional)</t>
-  </si>
-  <si>
-    <t>Nuclear_SMR</t>
-  </si>
-  <si>
-    <t>*HPS*,*hydro_ps*</t>
-  </si>
-  <si>
-    <t>Hydro_PS</t>
-  </si>
-  <si>
-    <t>Pumped Hydro Storage</t>
-  </si>
-  <si>
-    <t>Batt_Util</t>
-  </si>
-  <si>
-    <t>Utility Battery Storage</t>
-  </si>
-  <si>
-    <t>Batt_EV</t>
-  </si>
-  <si>
-    <t>EV Battery</t>
-  </si>
-  <si>
-    <t>EP_GAS-GT*,EP_OIL-GT*,*gas_turbine*,EN*CT*</t>
-  </si>
-  <si>
-    <t>EP_COA-ST*,EP_LIG-ST*,*-CFB*,*coal_subcritical*</t>
-  </si>
-  <si>
-    <t>co2captured,co2[_]*</t>
-  </si>
-  <si>
-    <t>CO2Captured</t>
-  </si>
-  <si>
-    <t>co2s[_]*</t>
-  </si>
-  <si>
-    <t>CO2Stored</t>
-  </si>
-  <si>
-    <t>ELC,e[_]*</t>
-  </si>
-  <si>
-    <t>Electricity</t>
-  </si>
-  <si>
-    <t>Nuclear_P</t>
-  </si>
-  <si>
-    <t>~tfm_psets</t>
-  </si>
-  <si>
-    <t>setname</t>
-  </si>
-  <si>
-    <t>pset_co</t>
-  </si>
-  <si>
-    <t>pset_ci</t>
-  </si>
-  <si>
-    <t>t_pos_andor</t>
-  </si>
-  <si>
-    <t>OR</t>
-  </si>
-  <si>
-    <t>-*ror*</t>
-  </si>
-  <si>
-    <t>EP_COA-SC*,EP_COA-USC*,EP_LIG-SC*,EP_LIG-USC*,*critical*</t>
-  </si>
-  <si>
-    <t>coal,elcco*</t>
-  </si>
-  <si>
-    <t>gas,elcnga,elcgas,oil,elco</t>
-  </si>
-  <si>
-    <t>bio*,elcb*</t>
-  </si>
-  <si>
-    <t>*HP*</t>
-  </si>
-  <si>
-    <t>-*HP*</t>
-  </si>
-  <si>
-    <t>elc,e[_]*</t>
-  </si>
-  <si>
-    <t>EP_GAS-IC*,EP_OIL-IC*,*gas_engine*,*internal_comb*</t>
-  </si>
-  <si>
-    <t>EP_GAS-CC*,EP_OIL-CC*,*gas_cc*,*gas_comb*,*ember</t>
-  </si>
-  <si>
-    <t>EP_GAS-ST*,EP_OIL-ST*,*steam*</t>
   </si>
   <si>
     <t>p_Artvin_TUR</t>
@@ -1231,8 +1228,8 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1260,9 +1257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1300,7 +1297,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1406,7 +1403,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1548,14 +1545,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1572,70 +1569,70 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="D7" t="str">
         <f>B7</f>
@@ -1644,7 +1641,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D8" t="str">
         <f>B8</f>
@@ -1653,7 +1650,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D9" t="str">
         <f>B9</f>
@@ -1662,47 +1659,47 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>140</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D15" t="str">
         <f>B15</f>
@@ -1711,50 +1708,47 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>135</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:D16">
-    <sortCondition ref="A5:A16"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9596CD-0528-4380-8F2D-D99C9A838BA1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B9:E117"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>142</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>144</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>146</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
@@ -1768,7 +1762,7 @@
         <v>160</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.45">
@@ -1782,7 +1776,7 @@
         <v>162</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.45">
@@ -1796,7 +1790,7 @@
         <v>164</v>
       </c>
       <c r="E13" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.45">
@@ -1810,7 +1804,7 @@
         <v>166</v>
       </c>
       <c r="E14" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.45">
@@ -1824,7 +1818,7 @@
         <v>168</v>
       </c>
       <c r="E15" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.45">
@@ -1838,7 +1832,7 @@
         <v>170</v>
       </c>
       <c r="E16" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.45">
@@ -1852,7 +1846,7 @@
         <v>172</v>
       </c>
       <c r="E17" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.45">
@@ -1866,7 +1860,7 @@
         <v>174</v>
       </c>
       <c r="E18" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.45">
@@ -1880,7 +1874,7 @@
         <v>176</v>
       </c>
       <c r="E19" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.45">
@@ -1894,7 +1888,7 @@
         <v>178</v>
       </c>
       <c r="E20" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.45">
@@ -1908,7 +1902,7 @@
         <v>180</v>
       </c>
       <c r="E21" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.45">
@@ -1922,7 +1916,7 @@
         <v>182</v>
       </c>
       <c r="E22" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.45">
@@ -1936,7 +1930,7 @@
         <v>184</v>
       </c>
       <c r="E23" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
@@ -1950,7 +1944,7 @@
         <v>186</v>
       </c>
       <c r="E24" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
@@ -1964,7 +1958,7 @@
         <v>188</v>
       </c>
       <c r="E25" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.45">
@@ -1978,7 +1972,7 @@
         <v>190</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.45">
@@ -1992,7 +1986,7 @@
         <v>192</v>
       </c>
       <c r="E27" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
@@ -2006,7 +2000,7 @@
         <v>194</v>
       </c>
       <c r="E28" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.45">
@@ -2020,7 +2014,7 @@
         <v>196</v>
       </c>
       <c r="E29" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.45">
@@ -2034,7 +2028,7 @@
         <v>198</v>
       </c>
       <c r="E30" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.45">
@@ -2048,7 +2042,7 @@
         <v>200</v>
       </c>
       <c r="E31" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.45">
@@ -2062,7 +2056,7 @@
         <v>202</v>
       </c>
       <c r="E32" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.45">
@@ -2076,7 +2070,7 @@
         <v>204</v>
       </c>
       <c r="E33" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.45">
@@ -2090,7 +2084,7 @@
         <v>206</v>
       </c>
       <c r="E34" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.45">
@@ -2104,7 +2098,7 @@
         <v>208</v>
       </c>
       <c r="E35" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.45">
@@ -2118,7 +2112,7 @@
         <v>210</v>
       </c>
       <c r="E36" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.45">
@@ -2132,7 +2126,7 @@
         <v>212</v>
       </c>
       <c r="E37" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.45">
@@ -2146,7 +2140,7 @@
         <v>214</v>
       </c>
       <c r="E38" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.45">
@@ -2160,7 +2154,7 @@
         <v>216</v>
       </c>
       <c r="E39" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.45">
@@ -2174,7 +2168,7 @@
         <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.45">
@@ -2188,7 +2182,7 @@
         <v>220</v>
       </c>
       <c r="E41" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.45">
@@ -2202,7 +2196,7 @@
         <v>222</v>
       </c>
       <c r="E42" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.45">
@@ -2216,7 +2210,7 @@
         <v>224</v>
       </c>
       <c r="E43" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.45">
@@ -2230,7 +2224,7 @@
         <v>226</v>
       </c>
       <c r="E44" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.45">
@@ -2244,7 +2238,7 @@
         <v>228</v>
       </c>
       <c r="E45" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.45">
@@ -2258,7 +2252,7 @@
         <v>230</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.45">
@@ -2272,7 +2266,7 @@
         <v>232</v>
       </c>
       <c r="E47" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.45">
@@ -2286,7 +2280,7 @@
         <v>234</v>
       </c>
       <c r="E48" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
@@ -2300,7 +2294,7 @@
         <v>236</v>
       </c>
       <c r="E49" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
@@ -2314,7 +2308,7 @@
         <v>238</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
@@ -2328,7 +2322,7 @@
         <v>240</v>
       </c>
       <c r="E51" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.45">
@@ -2342,7 +2336,7 @@
         <v>242</v>
       </c>
       <c r="E52" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
@@ -2356,7 +2350,7 @@
         <v>244</v>
       </c>
       <c r="E53" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
@@ -2370,7 +2364,7 @@
         <v>246</v>
       </c>
       <c r="E54" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
@@ -2384,7 +2378,7 @@
         <v>248</v>
       </c>
       <c r="E55" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.45">
@@ -2398,7 +2392,7 @@
         <v>250</v>
       </c>
       <c r="E56" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
@@ -2412,7 +2406,7 @@
         <v>252</v>
       </c>
       <c r="E57" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.45">
@@ -2426,7 +2420,7 @@
         <v>254</v>
       </c>
       <c r="E58" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.45">
@@ -2440,7 +2434,7 @@
         <v>256</v>
       </c>
       <c r="E59" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.45">
@@ -2454,7 +2448,7 @@
         <v>258</v>
       </c>
       <c r="E60" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.45">
@@ -2468,7 +2462,7 @@
         <v>260</v>
       </c>
       <c r="E61" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.45">
@@ -2482,7 +2476,7 @@
         <v>262</v>
       </c>
       <c r="E62" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.45">
@@ -2496,7 +2490,7 @@
         <v>264</v>
       </c>
       <c r="E63" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.45">
@@ -2510,7 +2504,7 @@
         <v>266</v>
       </c>
       <c r="E64" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
@@ -2524,7 +2518,7 @@
         <v>268</v>
       </c>
       <c r="E65" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
@@ -2538,7 +2532,7 @@
         <v>270</v>
       </c>
       <c r="E66" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.45">
@@ -2552,7 +2546,7 @@
         <v>272</v>
       </c>
       <c r="E67" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.45">
@@ -2566,7 +2560,7 @@
         <v>274</v>
       </c>
       <c r="E68" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.45">
@@ -2580,7 +2574,7 @@
         <v>276</v>
       </c>
       <c r="E69" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.45">
@@ -2594,7 +2588,7 @@
         <v>278</v>
       </c>
       <c r="E70" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.45">
@@ -2608,7 +2602,7 @@
         <v>280</v>
       </c>
       <c r="E71" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.45">
@@ -2622,7 +2616,7 @@
         <v>282</v>
       </c>
       <c r="E72" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.45">
@@ -2636,7 +2630,7 @@
         <v>284</v>
       </c>
       <c r="E73" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.45">
@@ -2650,7 +2644,7 @@
         <v>286</v>
       </c>
       <c r="E74" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.45">
@@ -2664,7 +2658,7 @@
         <v>288</v>
       </c>
       <c r="E75" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.45">
@@ -2678,7 +2672,7 @@
         <v>290</v>
       </c>
       <c r="E76" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.45">
@@ -2692,7 +2686,7 @@
         <v>292</v>
       </c>
       <c r="E77" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.45">
@@ -2706,7 +2700,7 @@
         <v>294</v>
       </c>
       <c r="E78" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.45">
@@ -2720,7 +2714,7 @@
         <v>296</v>
       </c>
       <c r="E79" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.45">
@@ -2734,7 +2728,7 @@
         <v>298</v>
       </c>
       <c r="E80" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.45">
@@ -2748,7 +2742,7 @@
         <v>300</v>
       </c>
       <c r="E81" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.45">
@@ -2762,7 +2756,7 @@
         <v>302</v>
       </c>
       <c r="E82" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.45">
@@ -2776,7 +2770,7 @@
         <v>304</v>
       </c>
       <c r="E83" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.45">
@@ -2790,7 +2784,7 @@
         <v>306</v>
       </c>
       <c r="E84" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.45">
@@ -2804,7 +2798,7 @@
         <v>308</v>
       </c>
       <c r="E85" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.45">
@@ -2818,7 +2812,7 @@
         <v>310</v>
       </c>
       <c r="E86" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.45">
@@ -2832,7 +2826,7 @@
         <v>312</v>
       </c>
       <c r="E87" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.45">
@@ -2846,7 +2840,7 @@
         <v>314</v>
       </c>
       <c r="E88" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.45">
@@ -2860,7 +2854,7 @@
         <v>316</v>
       </c>
       <c r="E89" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="90" spans="2:5" x14ac:dyDescent="0.45">
@@ -2874,7 +2868,7 @@
         <v>318</v>
       </c>
       <c r="E90" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.45">
@@ -2888,7 +2882,7 @@
         <v>320</v>
       </c>
       <c r="E91" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.45">
@@ -2902,7 +2896,7 @@
         <v>322</v>
       </c>
       <c r="E92" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.45">
@@ -2916,7 +2910,7 @@
         <v>324</v>
       </c>
       <c r="E93" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.45">
@@ -2930,7 +2924,7 @@
         <v>326</v>
       </c>
       <c r="E94" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.45">
@@ -2944,7 +2938,7 @@
         <v>328</v>
       </c>
       <c r="E95" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.45">
@@ -2958,7 +2952,7 @@
         <v>330</v>
       </c>
       <c r="E96" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.45">
@@ -2972,7 +2966,7 @@
         <v>332</v>
       </c>
       <c r="E97" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.45">
@@ -2986,7 +2980,7 @@
         <v>334</v>
       </c>
       <c r="E98" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.45">
@@ -3000,7 +2994,7 @@
         <v>336</v>
       </c>
       <c r="E99" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.45">
@@ -3014,7 +3008,7 @@
         <v>338</v>
       </c>
       <c r="E100" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.45">
@@ -3028,7 +3022,7 @@
         <v>340</v>
       </c>
       <c r="E101" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.45">
@@ -3042,7 +3036,7 @@
         <v>342</v>
       </c>
       <c r="E102" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.45">
@@ -3056,7 +3050,7 @@
         <v>344</v>
       </c>
       <c r="E103" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.45">
@@ -3070,7 +3064,7 @@
         <v>346</v>
       </c>
       <c r="E104" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.45">
@@ -3084,7 +3078,7 @@
         <v>348</v>
       </c>
       <c r="E105" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.45">
@@ -3098,7 +3092,7 @@
         <v>350</v>
       </c>
       <c r="E106" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.45">
@@ -3112,7 +3106,7 @@
         <v>352</v>
       </c>
       <c r="E107" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.45">
@@ -3126,7 +3120,7 @@
         <v>354</v>
       </c>
       <c r="E108" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.45">
@@ -3140,7 +3134,7 @@
         <v>356</v>
       </c>
       <c r="E109" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.45">
@@ -3154,7 +3148,7 @@
         <v>358</v>
       </c>
       <c r="E110" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.45">
@@ -3168,7 +3162,7 @@
         <v>360</v>
       </c>
       <c r="E111" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.45">
@@ -3182,7 +3176,7 @@
         <v>362</v>
       </c>
       <c r="E112" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.45">
@@ -3196,7 +3190,7 @@
         <v>364</v>
       </c>
       <c r="E113" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.45">
@@ -3210,7 +3204,7 @@
         <v>366</v>
       </c>
       <c r="E114" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.45">
@@ -3224,7 +3218,7 @@
         <v>368</v>
       </c>
       <c r="E115" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.45">
@@ -3238,7 +3232,7 @@
         <v>370</v>
       </c>
       <c r="E116" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="2:5" x14ac:dyDescent="0.45">
@@ -3252,7 +3246,7 @@
         <v>372</v>
       </c>
       <c r="E117" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -3261,7 +3255,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718D7FD7-C83A-40FD-B4D1-09885A1486FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -3277,561 +3271,561 @@
     <col min="10" max="10" width="24.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="H2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="G3" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="J4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="J7" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="J8" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="J10" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="G13" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>154</v>
+        <v>91</v>
       </c>
       <c r="D15" t="s">
-        <v>155</v>
+        <v>92</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="G15" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" t="s">
         <v>96</v>
       </c>
-      <c r="B16" t="s">
-        <v>153</v>
-      </c>
-      <c r="D16" t="s">
-        <v>155</v>
-      </c>
-      <c r="F16" t="s">
-        <v>103</v>
-      </c>
       <c r="G16" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D19" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F19" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G19" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D20" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="G20" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D21" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G21" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" t="s">
+        <v>115</v>
+      </c>
+      <c r="G22" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" t="s">
+        <v>117</v>
+      </c>
+      <c r="I22" t="s">
         <v>118</v>
-      </c>
-      <c r="F22" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" t="s">
-        <v>54</v>
-      </c>
-      <c r="H22" t="s">
-        <v>26</v>
-      </c>
-      <c r="I22" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" t="s">
         <v>120</v>
       </c>
-      <c r="D23" t="s">
-        <v>118</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>121</v>
-      </c>
-      <c r="G23" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
         <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="G24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="I24" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="D25" t="s">
         <v>123</v>
       </c>
       <c r="F25" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G25" t="s">
-        <v>51</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F26" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G26" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>133</v>
       </c>
       <c r="F27" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="G27" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H27" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="I27" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>136</v>
       </c>
       <c r="F28" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="G28" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A34" s="2" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="H34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>29</v>
+        <v>139</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="F35" t="s">
-        <v>28</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>31</v>
+        <v>142</v>
       </c>
       <c r="F36" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="B37" t="s">
-        <v>50</v>
+        <v>145</v>
       </c>
       <c r="F37" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="B38" t="s">
-        <v>61</v>
+        <v>147</v>
       </c>
       <c r="F38" t="s">
-        <v>62</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B39" t="s">
-        <v>65</v>
+        <v>149</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B40" t="s">
-        <v>59</v>
+        <v>151</v>
       </c>
       <c r="F40" t="s">
-        <v>60</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B41" t="s">
-        <v>67</v>
+        <v>153</v>
       </c>
       <c r="F41" s="3" t="str">
         <f>LEFT(B41,9)</f>
@@ -3840,25 +3834,25 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B42" t="s">
-        <v>68</v>
+        <v>154</v>
       </c>
       <c r="F42" s="3" t="str">
-        <f t="shared" ref="F42:F43" si="0">LEFT(B42,9)</f>
+        <f>LEFT(B42,9)</f>
         <v>distr_won</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
       <c r="F43" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>LEFT(B43,9)</f>
         <v>distr_wof</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D44" t="s">
-        <v>23</v>
+        <v>156</v>
       </c>
       <c r="F44" s="3" t="str">
         <f>"hs_"&amp;D44</f>
@@ -3867,28 +3861,28 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D45" t="s">
-        <v>24</v>
+        <v>157</v>
       </c>
       <c r="F45" s="3" t="str">
-        <f t="shared" ref="F45:F47" si="1">"hs_"&amp;D45</f>
+        <f>"hs_"&amp;D45</f>
         <v>hs_hydro</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D46" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F46" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>"hs_"&amp;D46</f>
         <v>hs_nuclear</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D47" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="F47" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>"hs_"&amp;D47</f>
         <v>hs_coal</v>
       </c>
     </row>

</xml_diff>